<commit_message>
feat: PDF de facturas, envío por mail/WhatsApp, email_cliente en Excel y BD
</commit_message>
<xml_diff>
--- a/app/static/plantilla_monotributo_masfacil.xlsx
+++ b/app/static/plantilla_monotributo_masfacil.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facturas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,17 +33,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002C3178"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00333333"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -71,7 +59,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -79,37 +67,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00DDDDDD"/>
-      </left>
-      <right style="thin">
-        <color rgb="00DDDDDD"/>
-      </right>
-      <top style="thin">
-        <color rgb="00DDDDDD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00DDDDDD"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,18 +443,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>fecha</t>
@@ -509,16 +478,21 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>email_cliente</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>concepto</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>monotributista</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>01/07/2026</t>
@@ -539,16 +513,21 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Honorarios julio 2026</t>
+          <t>juan@gmail.com</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Honorarios julio</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>García Silvana</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
+    <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>01/07/2026</t>
@@ -567,18 +546,19 @@
           <t>30-71234567-8</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Diseño web — julio</t>
-        </is>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
+          <t>Diseño web</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>García Silvana</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>01/07/2026</t>
@@ -599,190 +579,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Consultoría contable</t>
+          <t>ana@empresa.com</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Consultoría</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Rodríguez Pablo</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>15/07/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>120000</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Empresa SA</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>30-98765432-1</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Asesoramiento mes</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Rodríguez Pablo</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>MONOTRIBUTO MÁS FÁCIL — Plantilla de importación</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>COLUMNAS REQUERIDAS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • fecha          → Fecha de la factura. Formatos aceptados: DD/MM/YYYY o YYYY-MM-DD</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • importe        → Importe en pesos. Acepta: 50000, $50.000 o 50.000,00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • cliente        → Nombre completo del cliente que recibe la factura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • concepto       → Descripción del servicio (aparece en la factura)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • monotributista → Nombre o CUIT del monotributista que emite la factura</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>COLUMNAS OPCIONALES:</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • dni_cliente    → DNI (sin puntos) o CUIT (con o sin guiones) del cliente</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>TIPS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • El sistema reconoce automáticamente a cada monotributista por su nombre o CUIT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Si el cliente no existe, se crea automáticamente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Podés incluir múltiples monotributistas en el mismo Excel — se emiten en paralelo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Las filas con errores se saltan y se muestran en el preview antes de emitir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Las columnas pueden estar en cualquier orden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>SOPORTE:</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  📧 soporte@masfacil.com.ar</t>
         </is>
       </c>
     </row>

</xml_diff>